<commit_message>
feat: correção da estrutura de usuario
</commit_message>
<xml_diff>
--- a/usuario-api/Cadastro_em_Massa.xlsx
+++ b/usuario-api/Cadastro_em_Massa.xlsx
@@ -20,171 +20,168 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="83">
-  <si>
-    <t xml:space="preserve">Ana Silva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ana.silva@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">asilva</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adm@2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADMINISTRADOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruno Santos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bruno.santos@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bsantos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">User#123</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="82">
+  <si>
+    <t xml:space="preserve">Carlos Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlos.santos@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">csantos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlinhos</t>
   </si>
   <si>
     <t xml:space="preserve">USUARIO</t>
   </si>
   <si>
-    <t xml:space="preserve">Carla Oliveira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carla.oliveira@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coliveira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gerencia$99</t>
+    <t xml:space="preserve">Ana Rodrigues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ana.rodrigues@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arodrigues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aninha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pedro Oliveira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pedro.oliveira@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">poliveira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pepe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mariana Pereira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mariana.pereira@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mpereira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gabriel Lima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gabriel.lima@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">glima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrícia Fernandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">patricia.fernandes@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pfernandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiago Ramos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tiago.ramos@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tramos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ricardo Dias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ricardo.dias@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rdias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Isabela Costa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isabela.costa@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">icosta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bruno Ribeiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bruno.ribeiro@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bribeiro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brunão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fernanda Martins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fernanda.martins@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fmartins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lucas Alves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lucas.alves@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lalves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luc4s@lves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mariana Rocha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mariana.rocha@empresa.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mrocha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gestor@Mari</t>
   </si>
   <si>
     <t xml:space="preserve">GERENTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daniel Costa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">daniel.costa@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dcosta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dan@C0sta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduarda Pereira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eduarda.pereira@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epereira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teste1234</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabio Rodrigues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fabio.rodrigues@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">frodrigues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fab!o2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabriela Almeida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gabriela.almeida@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">galmeida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabi#User</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo Martins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hugo.martins@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hmartins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hm887766</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Isabela Ferreira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">isabela.ferreira@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">iferreira</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IsaFerra!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">João Souza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">joao.souza@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jsouza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuperAdm!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karina Lima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">karina.lima@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">klima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K@rinaL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lucas Alves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lucas.alves@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lalves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luc4s@lves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mariana Rocha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mariana.rocha@empresa.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mrocha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gestor@Mari</t>
   </si>
   <si>
     <t xml:space="preserve">Nicolas Mendes</t>
@@ -351,12 +348,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -553,351 +558,351 @@
   <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="B5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="B7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="E8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="E9" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="D12" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="B13" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="1" t="s">
+      <c r="C13" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="1" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="1" t="s">
+      <c r="B15" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="E15" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="B16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="E16" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+      <c r="B17" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="D17" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="E17" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E17" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
+      <c r="B18" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="C18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="E18" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E18" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+      <c r="B19" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="D19" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E19" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="D20" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>9</v>
+      <c r="E20" s="3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>